<commit_message>
Each model's performance with a patient-level 95% CI (Model Performance sheet)
</commit_message>
<xml_diff>
--- a/examples/example_classifier_results.xlsx
+++ b/examples/example_classifier_results.xlsx
@@ -9,15 +9,16 @@
   <sheets>
     <sheet name="Results" sheetId="1" r:id="rId1"/>
     <sheet name="Statistical Tests" sheetId="2" r:id="rId2"/>
-    <sheet name="Estimates" sheetId="3" r:id="rId3"/>
-    <sheet name="Sample" sheetId="4" r:id="rId4"/>
+    <sheet name="Model Performance" sheetId="3" r:id="rId3"/>
+    <sheet name="Estimates" sheetId="4" r:id="rId4"/>
+    <sheet name="Sample" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="635" uniqueCount="110">
   <si>
     <t>Group</t>
   </si>
@@ -202,15 +203,60 @@
     <t>Romano-Wolf (bootstrap tests) / Hommel (other tests)</t>
   </si>
   <si>
-    <t>rho_delta: intraclass correlation of the per-eye difference in loss between the two models; one_eye_factor: patients a one-eye study needs, relative to this analysis (design effect)</t>
+    <t>ρΔ (rho_delta): intraclass correlation of the per-eye difference in loss between the two models; one_eye_factor: patients a one-eye study needs, relative to this analysis (design effect)</t>
   </si>
   <si>
     <t>group</t>
   </si>
   <si>
+    <t>model</t>
+  </si>
+  <si>
     <t>metric</t>
   </si>
   <si>
+    <t>estimate</t>
+  </si>
+  <si>
+    <t>ci_low</t>
+  </si>
+  <si>
+    <t>ci_high</t>
+  </si>
+  <si>
+    <t>n_eyes</t>
+  </si>
+  <si>
+    <t>n_patients</t>
+  </si>
+  <si>
+    <t>method</t>
+  </si>
+  <si>
+    <t>auc</t>
+  </si>
+  <si>
+    <t>brier</t>
+  </si>
+  <si>
+    <t>logloss</t>
+  </si>
+  <si>
+    <t>sensitivity</t>
+  </si>
+  <si>
+    <t>specificity</t>
+  </si>
+  <si>
+    <t>accuracy</t>
+  </si>
+  <si>
+    <t>patient bootstrap, percentile</t>
+  </si>
+  <si>
+    <t>bootstrap, percentile</t>
+  </si>
+  <si>
     <t>model_a</t>
   </si>
   <si>
@@ -226,12 +272,6 @@
     <t>diff</t>
   </si>
   <si>
-    <t>ci_low</t>
-  </si>
-  <si>
-    <t>ci_high</t>
-  </si>
-  <si>
     <t>p</t>
   </si>
   <si>
@@ -247,24 +287,6 @@
     <t>p_adj</t>
   </si>
   <si>
-    <t>auc</t>
-  </si>
-  <si>
-    <t>brier</t>
-  </si>
-  <si>
-    <t>logloss</t>
-  </si>
-  <si>
-    <t>sensitivity</t>
-  </si>
-  <si>
-    <t>specificity</t>
-  </si>
-  <si>
-    <t>accuracy</t>
-  </si>
-  <si>
     <t>DeLong (1988)</t>
   </si>
   <si>
@@ -281,12 +303,6 @@
   </si>
   <si>
     <t>truth</t>
-  </si>
-  <si>
-    <t>n_eyes</t>
-  </si>
-  <si>
-    <t>n_patients</t>
   </si>
   <si>
     <t>n_bilateral</t>
@@ -1867,6 +1883,1614 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I55"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="9" width="18.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E1" t="s">
+        <v>66</v>
+      </c>
+      <c r="F1" t="s">
+        <v>67</v>
+      </c>
+      <c r="G1" t="s">
+        <v>68</v>
+      </c>
+      <c r="H1" t="s">
+        <v>69</v>
+      </c>
+      <c r="I1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D2">
+        <v>0.9497450348899624</v>
+      </c>
+      <c r="E2">
+        <v>0.9320893216905599</v>
+      </c>
+      <c r="F2">
+        <v>0.9658422111533366</v>
+      </c>
+      <c r="G2">
+        <v>516</v>
+      </c>
+      <c r="H2">
+        <v>300</v>
+      </c>
+      <c r="I2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" t="s">
+        <v>71</v>
+      </c>
+      <c r="D3">
+        <v>0.9360670194003528</v>
+      </c>
+      <c r="E3">
+        <v>0.9132995820124723</v>
+      </c>
+      <c r="F3">
+        <v>0.9561922327746769</v>
+      </c>
+      <c r="G3">
+        <v>516</v>
+      </c>
+      <c r="H3">
+        <v>300</v>
+      </c>
+      <c r="I3" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C4" t="s">
+        <v>71</v>
+      </c>
+      <c r="D4">
+        <v>0.888888888888889</v>
+      </c>
+      <c r="E4">
+        <v>0.8573046968123558</v>
+      </c>
+      <c r="F4">
+        <v>0.9177145234366175</v>
+      </c>
+      <c r="G4">
+        <v>516</v>
+      </c>
+      <c r="H4">
+        <v>300</v>
+      </c>
+      <c r="I4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C5" t="s">
+        <v>72</v>
+      </c>
+      <c r="D5">
+        <v>0.09039919269379845</v>
+      </c>
+      <c r="E5">
+        <v>0.07832652244405816</v>
+      </c>
+      <c r="F5">
+        <v>0.1022662245047647</v>
+      </c>
+      <c r="G5">
+        <v>516</v>
+      </c>
+      <c r="H5">
+        <v>300</v>
+      </c>
+      <c r="I5" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" t="s">
+        <v>72</v>
+      </c>
+      <c r="D6">
+        <v>0.09607086470930232</v>
+      </c>
+      <c r="E6">
+        <v>0.08251477675096154</v>
+      </c>
+      <c r="F6">
+        <v>0.1101717326762754</v>
+      </c>
+      <c r="G6">
+        <v>516</v>
+      </c>
+      <c r="H6">
+        <v>300</v>
+      </c>
+      <c r="I6" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" t="s">
+        <v>72</v>
+      </c>
+      <c r="D7">
+        <v>0.1235763627906977</v>
+      </c>
+      <c r="E7">
+        <v>0.1064186137780775</v>
+      </c>
+      <c r="F7">
+        <v>0.1410180048162069</v>
+      </c>
+      <c r="G7">
+        <v>516</v>
+      </c>
+      <c r="H7">
+        <v>300</v>
+      </c>
+      <c r="I7" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" t="s">
+        <v>38</v>
+      </c>
+      <c r="C8" t="s">
+        <v>73</v>
+      </c>
+      <c r="D8">
+        <v>0.3017094343669053</v>
+      </c>
+      <c r="E8">
+        <v>0.2707681375493131</v>
+      </c>
+      <c r="F8">
+        <v>0.3317168115905306</v>
+      </c>
+      <c r="G8">
+        <v>516</v>
+      </c>
+      <c r="H8">
+        <v>300</v>
+      </c>
+      <c r="I8" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" t="s">
+        <v>39</v>
+      </c>
+      <c r="C9" t="s">
+        <v>73</v>
+      </c>
+      <c r="D9">
+        <v>0.3154288386745746</v>
+      </c>
+      <c r="E9">
+        <v>0.2813931137035998</v>
+      </c>
+      <c r="F9">
+        <v>0.3510561699111525</v>
+      </c>
+      <c r="G9">
+        <v>516</v>
+      </c>
+      <c r="H9">
+        <v>300</v>
+      </c>
+      <c r="I9" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" t="s">
+        <v>73</v>
+      </c>
+      <c r="D10">
+        <v>0.3822401917568288</v>
+      </c>
+      <c r="E10">
+        <v>0.3387446684060572</v>
+      </c>
+      <c r="F10">
+        <v>0.4265781353425924</v>
+      </c>
+      <c r="G10">
+        <v>516</v>
+      </c>
+      <c r="H10">
+        <v>300</v>
+      </c>
+      <c r="I10" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11" t="s">
+        <v>74</v>
+      </c>
+      <c r="D11">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="E11">
+        <v>0.7656013257575758</v>
+      </c>
+      <c r="F11">
+        <v>0.8960148148148149</v>
+      </c>
+      <c r="G11">
+        <v>516</v>
+      </c>
+      <c r="H11">
+        <v>300</v>
+      </c>
+      <c r="I11" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" t="s">
+        <v>35</v>
+      </c>
+      <c r="B12" t="s">
+        <v>39</v>
+      </c>
+      <c r="C12" t="s">
+        <v>74</v>
+      </c>
+      <c r="D12">
+        <v>0.8043478260869565</v>
+      </c>
+      <c r="E12">
+        <v>0.7333333333333333</v>
+      </c>
+      <c r="F12">
+        <v>0.8695652173913043</v>
+      </c>
+      <c r="G12">
+        <v>516</v>
+      </c>
+      <c r="H12">
+        <v>300</v>
+      </c>
+      <c r="I12" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" t="s">
+        <v>74</v>
+      </c>
+      <c r="D13">
+        <v>0.7608695652173914</v>
+      </c>
+      <c r="E13">
+        <v>0.6846128033040785</v>
+      </c>
+      <c r="F13">
+        <v>0.8333333333333334</v>
+      </c>
+      <c r="G13">
+        <v>516</v>
+      </c>
+      <c r="H13">
+        <v>300</v>
+      </c>
+      <c r="I13" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" t="s">
+        <v>35</v>
+      </c>
+      <c r="B14" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" t="s">
+        <v>75</v>
+      </c>
+      <c r="D14">
+        <v>0.8862433862433863</v>
+      </c>
+      <c r="E14">
+        <v>0.852937169418176</v>
+      </c>
+      <c r="F14">
+        <v>0.9182058047493403</v>
+      </c>
+      <c r="G14">
+        <v>516</v>
+      </c>
+      <c r="H14">
+        <v>300</v>
+      </c>
+      <c r="I14" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15" t="s">
+        <v>35</v>
+      </c>
+      <c r="B15" t="s">
+        <v>39</v>
+      </c>
+      <c r="C15" t="s">
+        <v>75</v>
+      </c>
+      <c r="D15">
+        <v>0.8994708994708994</v>
+      </c>
+      <c r="E15">
+        <v>0.8660881121774977</v>
+      </c>
+      <c r="F15">
+        <v>0.9300518134715026</v>
+      </c>
+      <c r="G15">
+        <v>516</v>
+      </c>
+      <c r="H15">
+        <v>300</v>
+      </c>
+      <c r="I15" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" t="s">
+        <v>40</v>
+      </c>
+      <c r="C16" t="s">
+        <v>75</v>
+      </c>
+      <c r="D16">
+        <v>0.8465608465608465</v>
+      </c>
+      <c r="E16">
+        <v>0.8077940861367046</v>
+      </c>
+      <c r="F16">
+        <v>0.8837240729101195</v>
+      </c>
+      <c r="G16">
+        <v>516</v>
+      </c>
+      <c r="H16">
+        <v>300</v>
+      </c>
+      <c r="I16" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17" t="s">
+        <v>38</v>
+      </c>
+      <c r="C17" t="s">
+        <v>76</v>
+      </c>
+      <c r="D17">
+        <v>0.8720930232558139</v>
+      </c>
+      <c r="E17">
+        <v>0.8428290766208252</v>
+      </c>
+      <c r="F17">
+        <v>0.9011928958756779</v>
+      </c>
+      <c r="G17">
+        <v>516</v>
+      </c>
+      <c r="H17">
+        <v>300</v>
+      </c>
+      <c r="I17" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" t="s">
+        <v>35</v>
+      </c>
+      <c r="B18" t="s">
+        <v>39</v>
+      </c>
+      <c r="C18" t="s">
+        <v>76</v>
+      </c>
+      <c r="D18">
+        <v>0.874031007751938</v>
+      </c>
+      <c r="E18">
+        <v>0.8448275862068966</v>
+      </c>
+      <c r="F18">
+        <v>0.9020735511528966</v>
+      </c>
+      <c r="G18">
+        <v>516</v>
+      </c>
+      <c r="H18">
+        <v>300</v>
+      </c>
+      <c r="I18" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="A19" t="s">
+        <v>35</v>
+      </c>
+      <c r="B19" t="s">
+        <v>40</v>
+      </c>
+      <c r="C19" t="s">
+        <v>76</v>
+      </c>
+      <c r="D19">
+        <v>0.8236434108527132</v>
+      </c>
+      <c r="E19">
+        <v>0.7895702093070514</v>
+      </c>
+      <c r="F19">
+        <v>0.8568627450980392</v>
+      </c>
+      <c r="G19">
+        <v>516</v>
+      </c>
+      <c r="H19">
+        <v>300</v>
+      </c>
+      <c r="I19" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9">
+      <c r="A20" t="s">
+        <v>36</v>
+      </c>
+      <c r="B20" t="s">
+        <v>38</v>
+      </c>
+      <c r="C20" t="s">
+        <v>71</v>
+      </c>
+      <c r="D20">
+        <v>0.9572425828970333</v>
+      </c>
+      <c r="E20">
+        <v>0.9314174085184896</v>
+      </c>
+      <c r="F20">
+        <v>0.9779403804253587</v>
+      </c>
+      <c r="G20">
+        <v>263</v>
+      </c>
+      <c r="H20">
+        <v>263</v>
+      </c>
+      <c r="I20" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21" t="s">
+        <v>36</v>
+      </c>
+      <c r="B21" t="s">
+        <v>39</v>
+      </c>
+      <c r="C21" t="s">
+        <v>71</v>
+      </c>
+      <c r="D21">
+        <v>0.954261198371146</v>
+      </c>
+      <c r="E21">
+        <v>0.9278557781439901</v>
+      </c>
+      <c r="F21">
+        <v>0.9757148084114029</v>
+      </c>
+      <c r="G21">
+        <v>263</v>
+      </c>
+      <c r="H21">
+        <v>263</v>
+      </c>
+      <c r="I21" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22" t="s">
+        <v>36</v>
+      </c>
+      <c r="B22" t="s">
+        <v>40</v>
+      </c>
+      <c r="C22" t="s">
+        <v>71</v>
+      </c>
+      <c r="D22">
+        <v>0.9070680628272252</v>
+      </c>
+      <c r="E22">
+        <v>0.8680864992881939</v>
+      </c>
+      <c r="F22">
+        <v>0.9400875480541542</v>
+      </c>
+      <c r="G22">
+        <v>263</v>
+      </c>
+      <c r="H22">
+        <v>263</v>
+      </c>
+      <c r="I22" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9">
+      <c r="A23" t="s">
+        <v>36</v>
+      </c>
+      <c r="B23" t="s">
+        <v>38</v>
+      </c>
+      <c r="C23" t="s">
+        <v>72</v>
+      </c>
+      <c r="D23">
+        <v>0.08409677600760457</v>
+      </c>
+      <c r="E23">
+        <v>0.06911136540874524</v>
+      </c>
+      <c r="F23">
+        <v>0.1009847289695818</v>
+      </c>
+      <c r="G23">
+        <v>263</v>
+      </c>
+      <c r="H23">
+        <v>263</v>
+      </c>
+      <c r="I23" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9">
+      <c r="A24" t="s">
+        <v>36</v>
+      </c>
+      <c r="B24" t="s">
+        <v>39</v>
+      </c>
+      <c r="C24" t="s">
+        <v>72</v>
+      </c>
+      <c r="D24">
+        <v>0.08091932330798481</v>
+      </c>
+      <c r="E24">
+        <v>0.06420706836501901</v>
+      </c>
+      <c r="F24">
+        <v>0.09966024858365012</v>
+      </c>
+      <c r="G24">
+        <v>263</v>
+      </c>
+      <c r="H24">
+        <v>263</v>
+      </c>
+      <c r="I24" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9">
+      <c r="A25" t="s">
+        <v>36</v>
+      </c>
+      <c r="B25" t="s">
+        <v>40</v>
+      </c>
+      <c r="C25" t="s">
+        <v>72</v>
+      </c>
+      <c r="D25">
+        <v>0.1173666533840304</v>
+      </c>
+      <c r="E25">
+        <v>0.0959141370114068</v>
+      </c>
+      <c r="F25">
+        <v>0.1397679711159696</v>
+      </c>
+      <c r="G25">
+        <v>263</v>
+      </c>
+      <c r="H25">
+        <v>263</v>
+      </c>
+      <c r="I25" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9">
+      <c r="A26" t="s">
+        <v>36</v>
+      </c>
+      <c r="B26" t="s">
+        <v>38</v>
+      </c>
+      <c r="C26" t="s">
+        <v>73</v>
+      </c>
+      <c r="D26">
+        <v>0.2869453687617093</v>
+      </c>
+      <c r="E26">
+        <v>0.2491849800219261</v>
+      </c>
+      <c r="F26">
+        <v>0.3292138341683321</v>
+      </c>
+      <c r="G26">
+        <v>263</v>
+      </c>
+      <c r="H26">
+        <v>263</v>
+      </c>
+      <c r="I26" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9">
+      <c r="A27" t="s">
+        <v>36</v>
+      </c>
+      <c r="B27" t="s">
+        <v>39</v>
+      </c>
+      <c r="C27" t="s">
+        <v>73</v>
+      </c>
+      <c r="D27">
+        <v>0.2760765501167315</v>
+      </c>
+      <c r="E27">
+        <v>0.2337866905120009</v>
+      </c>
+      <c r="F27">
+        <v>0.3225826966370221</v>
+      </c>
+      <c r="G27">
+        <v>263</v>
+      </c>
+      <c r="H27">
+        <v>263</v>
+      </c>
+      <c r="I27" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9">
+      <c r="A28" t="s">
+        <v>36</v>
+      </c>
+      <c r="B28" t="s">
+        <v>40</v>
+      </c>
+      <c r="C28" t="s">
+        <v>73</v>
+      </c>
+      <c r="D28">
+        <v>0.3615170226541689</v>
+      </c>
+      <c r="E28">
+        <v>0.3096911889090577</v>
+      </c>
+      <c r="F28">
+        <v>0.4159065315200386</v>
+      </c>
+      <c r="G28">
+        <v>263</v>
+      </c>
+      <c r="H28">
+        <v>263</v>
+      </c>
+      <c r="I28" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9">
+      <c r="A29" t="s">
+        <v>36</v>
+      </c>
+      <c r="B29" t="s">
+        <v>38</v>
+      </c>
+      <c r="C29" t="s">
+        <v>74</v>
+      </c>
+      <c r="D29">
+        <v>0.8194444444444444</v>
+      </c>
+      <c r="E29">
+        <v>0.7241379310344828</v>
+      </c>
+      <c r="F29">
+        <v>0.9058823529411765</v>
+      </c>
+      <c r="G29">
+        <v>263</v>
+      </c>
+      <c r="H29">
+        <v>263</v>
+      </c>
+      <c r="I29" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9">
+      <c r="A30" t="s">
+        <v>36</v>
+      </c>
+      <c r="B30" t="s">
+        <v>39</v>
+      </c>
+      <c r="C30" t="s">
+        <v>74</v>
+      </c>
+      <c r="D30">
+        <v>0.8055555555555556</v>
+      </c>
+      <c r="E30">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="F30">
+        <v>0.8889649923896501</v>
+      </c>
+      <c r="G30">
+        <v>263</v>
+      </c>
+      <c r="H30">
+        <v>263</v>
+      </c>
+      <c r="I30" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9">
+      <c r="A31" t="s">
+        <v>36</v>
+      </c>
+      <c r="B31" t="s">
+        <v>40</v>
+      </c>
+      <c r="C31" t="s">
+        <v>74</v>
+      </c>
+      <c r="D31">
+        <v>0.7777777777777778</v>
+      </c>
+      <c r="E31">
+        <v>0.676056338028169</v>
+      </c>
+      <c r="F31">
+        <v>0.8676470588235294</v>
+      </c>
+      <c r="G31">
+        <v>263</v>
+      </c>
+      <c r="H31">
+        <v>263</v>
+      </c>
+      <c r="I31" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9">
+      <c r="A32" t="s">
+        <v>36</v>
+      </c>
+      <c r="B32" t="s">
+        <v>38</v>
+      </c>
+      <c r="C32" t="s">
+        <v>75</v>
+      </c>
+      <c r="D32">
+        <v>0.9057591623036649</v>
+      </c>
+      <c r="E32">
+        <v>0.8628515406162466</v>
+      </c>
+      <c r="F32">
+        <v>0.945273631840796</v>
+      </c>
+      <c r="G32">
+        <v>263</v>
+      </c>
+      <c r="H32">
+        <v>263</v>
+      </c>
+      <c r="I32" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9">
+      <c r="A33" t="s">
+        <v>36</v>
+      </c>
+      <c r="B33" t="s">
+        <v>39</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33">
+        <v>0.9162303664921466</v>
+      </c>
+      <c r="E33">
+        <v>0.8743455497382199</v>
+      </c>
+      <c r="F33">
+        <v>0.953223949337939</v>
+      </c>
+      <c r="G33">
+        <v>263</v>
+      </c>
+      <c r="H33">
+        <v>263</v>
+      </c>
+      <c r="I33" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9">
+      <c r="A34" t="s">
+        <v>36</v>
+      </c>
+      <c r="B34" t="s">
+        <v>40</v>
+      </c>
+      <c r="C34" t="s">
+        <v>75</v>
+      </c>
+      <c r="D34">
+        <v>0.837696335078534</v>
+      </c>
+      <c r="E34">
+        <v>0.7857142857142857</v>
+      </c>
+      <c r="F34">
+        <v>0.8888888888888888</v>
+      </c>
+      <c r="G34">
+        <v>263</v>
+      </c>
+      <c r="H34">
+        <v>263</v>
+      </c>
+      <c r="I34" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9">
+      <c r="A35" t="s">
+        <v>36</v>
+      </c>
+      <c r="B35" t="s">
+        <v>38</v>
+      </c>
+      <c r="C35" t="s">
+        <v>76</v>
+      </c>
+      <c r="D35">
+        <v>0.8821292775665399</v>
+      </c>
+      <c r="E35">
+        <v>0.8403041825095057</v>
+      </c>
+      <c r="F35">
+        <v>0.9201520912547528</v>
+      </c>
+      <c r="G35">
+        <v>263</v>
+      </c>
+      <c r="H35">
+        <v>263</v>
+      </c>
+      <c r="I35" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9">
+      <c r="A36" t="s">
+        <v>36</v>
+      </c>
+      <c r="B36" t="s">
+        <v>39</v>
+      </c>
+      <c r="C36" t="s">
+        <v>76</v>
+      </c>
+      <c r="D36">
+        <v>0.8859315589353612</v>
+      </c>
+      <c r="E36">
+        <v>0.844106463878327</v>
+      </c>
+      <c r="F36">
+        <v>0.9201520912547528</v>
+      </c>
+      <c r="G36">
+        <v>263</v>
+      </c>
+      <c r="H36">
+        <v>263</v>
+      </c>
+      <c r="I36" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9">
+      <c r="A37" t="s">
+        <v>36</v>
+      </c>
+      <c r="B37" t="s">
+        <v>40</v>
+      </c>
+      <c r="C37" t="s">
+        <v>76</v>
+      </c>
+      <c r="D37">
+        <v>0.8212927756653993</v>
+      </c>
+      <c r="E37">
+        <v>0.7756653992395437</v>
+      </c>
+      <c r="F37">
+        <v>0.8669201520912547</v>
+      </c>
+      <c r="G37">
+        <v>263</v>
+      </c>
+      <c r="H37">
+        <v>263</v>
+      </c>
+      <c r="I37" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9">
+      <c r="A38" t="s">
+        <v>37</v>
+      </c>
+      <c r="B38" t="s">
+        <v>38</v>
+      </c>
+      <c r="C38" t="s">
+        <v>71</v>
+      </c>
+      <c r="D38">
+        <v>0.9407308377896613</v>
+      </c>
+      <c r="E38">
+        <v>0.911409306760217</v>
+      </c>
+      <c r="F38">
+        <v>0.9649602719005704</v>
+      </c>
+      <c r="G38">
+        <v>253</v>
+      </c>
+      <c r="H38">
+        <v>253</v>
+      </c>
+      <c r="I38" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9">
+      <c r="A39" t="s">
+        <v>37</v>
+      </c>
+      <c r="B39" t="s">
+        <v>39</v>
+      </c>
+      <c r="C39" t="s">
+        <v>71</v>
+      </c>
+      <c r="D39">
+        <v>0.9163830821584832</v>
+      </c>
+      <c r="E39">
+        <v>0.8794413082083586</v>
+      </c>
+      <c r="F39">
+        <v>0.9491267011035582</v>
+      </c>
+      <c r="G39">
+        <v>253</v>
+      </c>
+      <c r="H39">
+        <v>253</v>
+      </c>
+      <c r="I39" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9">
+      <c r="A40" t="s">
+        <v>37</v>
+      </c>
+      <c r="B40" t="s">
+        <v>40</v>
+      </c>
+      <c r="C40" t="s">
+        <v>71</v>
+      </c>
+      <c r="D40">
+        <v>0.8704423918327662</v>
+      </c>
+      <c r="E40">
+        <v>0.8206890454828421</v>
+      </c>
+      <c r="F40">
+        <v>0.9151523253929671</v>
+      </c>
+      <c r="G40">
+        <v>253</v>
+      </c>
+      <c r="H40">
+        <v>253</v>
+      </c>
+      <c r="I40" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9">
+      <c r="A41" t="s">
+        <v>37</v>
+      </c>
+      <c r="B41" t="s">
+        <v>38</v>
+      </c>
+      <c r="C41" t="s">
+        <v>72</v>
+      </c>
+      <c r="D41">
+        <v>0.09695071675889329</v>
+      </c>
+      <c r="E41">
+        <v>0.08017872622529643</v>
+      </c>
+      <c r="F41">
+        <v>0.1154392034308301</v>
+      </c>
+      <c r="G41">
+        <v>253</v>
+      </c>
+      <c r="H41">
+        <v>253</v>
+      </c>
+      <c r="I41" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9">
+      <c r="A42" t="s">
+        <v>37</v>
+      </c>
+      <c r="B42" t="s">
+        <v>39</v>
+      </c>
+      <c r="C42" t="s">
+        <v>72</v>
+      </c>
+      <c r="D42">
+        <v>0.1118212812648221</v>
+      </c>
+      <c r="E42">
+        <v>0.0916886461521739</v>
+      </c>
+      <c r="F42">
+        <v>0.1326395123577075</v>
+      </c>
+      <c r="G42">
+        <v>253</v>
+      </c>
+      <c r="H42">
+        <v>253</v>
+      </c>
+      <c r="I42" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9">
+      <c r="A43" t="s">
+        <v>37</v>
+      </c>
+      <c r="B43" t="s">
+        <v>40</v>
+      </c>
+      <c r="C43" t="s">
+        <v>72</v>
+      </c>
+      <c r="D43">
+        <v>0.130031515256917</v>
+      </c>
+      <c r="E43">
+        <v>0.1057446896225297</v>
+      </c>
+      <c r="F43">
+        <v>0.1559957030592885</v>
+      </c>
+      <c r="G43">
+        <v>253</v>
+      </c>
+      <c r="H43">
+        <v>253</v>
+      </c>
+      <c r="I43" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9">
+      <c r="A44" t="s">
+        <v>37</v>
+      </c>
+      <c r="B44" t="s">
+        <v>38</v>
+      </c>
+      <c r="C44" t="s">
+        <v>73</v>
+      </c>
+      <c r="D44">
+        <v>0.317057059877445</v>
+      </c>
+      <c r="E44">
+        <v>0.2758562403397774</v>
+      </c>
+      <c r="F44">
+        <v>0.3622894928340787</v>
+      </c>
+      <c r="G44">
+        <v>253</v>
+      </c>
+      <c r="H44">
+        <v>253</v>
+      </c>
+      <c r="I44" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9">
+      <c r="A45" t="s">
+        <v>37</v>
+      </c>
+      <c r="B45" t="s">
+        <v>39</v>
+      </c>
+      <c r="C45" t="s">
+        <v>73</v>
+      </c>
+      <c r="D45">
+        <v>0.3563365536576291</v>
+      </c>
+      <c r="E45">
+        <v>0.3056173165279735</v>
+      </c>
+      <c r="F45">
+        <v>0.4092161441083348</v>
+      </c>
+      <c r="G45">
+        <v>253</v>
+      </c>
+      <c r="H45">
+        <v>253</v>
+      </c>
+      <c r="I45" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9">
+      <c r="A46" t="s">
+        <v>37</v>
+      </c>
+      <c r="B46" t="s">
+        <v>40</v>
+      </c>
+      <c r="C46" t="s">
+        <v>73</v>
+      </c>
+      <c r="D46">
+        <v>0.4037824584524792</v>
+      </c>
+      <c r="E46">
+        <v>0.3398855733723783</v>
+      </c>
+      <c r="F46">
+        <v>0.4722873582532369</v>
+      </c>
+      <c r="G46">
+        <v>253</v>
+      </c>
+      <c r="H46">
+        <v>253</v>
+      </c>
+      <c r="I46" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9">
+      <c r="A47" t="s">
+        <v>37</v>
+      </c>
+      <c r="B47" t="s">
+        <v>38</v>
+      </c>
+      <c r="C47" t="s">
+        <v>74</v>
+      </c>
+      <c r="D47">
+        <v>0.8484848484848485</v>
+      </c>
+      <c r="E47">
+        <v>0.7534246575342466</v>
+      </c>
+      <c r="F47">
+        <v>0.9305555555555556</v>
+      </c>
+      <c r="G47">
+        <v>253</v>
+      </c>
+      <c r="H47">
+        <v>253</v>
+      </c>
+      <c r="I47" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9">
+      <c r="A48" t="s">
+        <v>37</v>
+      </c>
+      <c r="B48" t="s">
+        <v>39</v>
+      </c>
+      <c r="C48" t="s">
+        <v>74</v>
+      </c>
+      <c r="D48">
+        <v>0.803030303030303</v>
+      </c>
+      <c r="E48">
+        <v>0.7017543859649122</v>
+      </c>
+      <c r="F48">
+        <v>0.8947368421052632</v>
+      </c>
+      <c r="G48">
+        <v>253</v>
+      </c>
+      <c r="H48">
+        <v>253</v>
+      </c>
+      <c r="I48" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9">
+      <c r="A49" t="s">
+        <v>37</v>
+      </c>
+      <c r="B49" t="s">
+        <v>40</v>
+      </c>
+      <c r="C49" t="s">
+        <v>74</v>
+      </c>
+      <c r="D49">
+        <v>0.7424242424242424</v>
+      </c>
+      <c r="E49">
+        <v>0.6323529411764706</v>
+      </c>
+      <c r="F49">
+        <v>0.8450704225352113</v>
+      </c>
+      <c r="G49">
+        <v>253</v>
+      </c>
+      <c r="H49">
+        <v>253</v>
+      </c>
+      <c r="I49" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9">
+      <c r="A50" t="s">
+        <v>37</v>
+      </c>
+      <c r="B50" t="s">
+        <v>38</v>
+      </c>
+      <c r="C50" t="s">
+        <v>75</v>
+      </c>
+      <c r="D50">
+        <v>0.8663101604278075</v>
+      </c>
+      <c r="E50">
+        <v>0.8148044111527257</v>
+      </c>
+      <c r="F50">
+        <v>0.9135135135135135</v>
+      </c>
+      <c r="G50">
+        <v>253</v>
+      </c>
+      <c r="H50">
+        <v>253</v>
+      </c>
+      <c r="I50" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9">
+      <c r="A51" t="s">
+        <v>37</v>
+      </c>
+      <c r="B51" t="s">
+        <v>39</v>
+      </c>
+      <c r="C51" t="s">
+        <v>75</v>
+      </c>
+      <c r="D51">
+        <v>0.8823529411764706</v>
+      </c>
+      <c r="E51">
+        <v>0.835046541887699</v>
+      </c>
+      <c r="F51">
+        <v>0.9259259259259259</v>
+      </c>
+      <c r="G51">
+        <v>253</v>
+      </c>
+      <c r="H51">
+        <v>253</v>
+      </c>
+      <c r="I51" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9">
+      <c r="A52" t="s">
+        <v>37</v>
+      </c>
+      <c r="B52" t="s">
+        <v>40</v>
+      </c>
+      <c r="C52" t="s">
+        <v>75</v>
+      </c>
+      <c r="D52">
+        <v>0.8556149732620321</v>
+      </c>
+      <c r="E52">
+        <v>0.8011363636363636</v>
+      </c>
+      <c r="F52">
+        <v>0.9039590823489129</v>
+      </c>
+      <c r="G52">
+        <v>253</v>
+      </c>
+      <c r="H52">
+        <v>253</v>
+      </c>
+      <c r="I52" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9">
+      <c r="A53" t="s">
+        <v>37</v>
+      </c>
+      <c r="B53" t="s">
+        <v>38</v>
+      </c>
+      <c r="C53" t="s">
+        <v>76</v>
+      </c>
+      <c r="D53">
+        <v>0.8616600790513834</v>
+      </c>
+      <c r="E53">
+        <v>0.8181818181818182</v>
+      </c>
+      <c r="F53">
+        <v>0.9011857707509882</v>
+      </c>
+      <c r="G53">
+        <v>253</v>
+      </c>
+      <c r="H53">
+        <v>253</v>
+      </c>
+      <c r="I53" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9">
+      <c r="A54" t="s">
+        <v>37</v>
+      </c>
+      <c r="B54" t="s">
+        <v>39</v>
+      </c>
+      <c r="C54" t="s">
+        <v>76</v>
+      </c>
+      <c r="D54">
+        <v>0.8616600790513834</v>
+      </c>
+      <c r="E54">
+        <v>0.8181818181818182</v>
+      </c>
+      <c r="F54">
+        <v>0.9011857707509882</v>
+      </c>
+      <c r="G54">
+        <v>253</v>
+      </c>
+      <c r="H54">
+        <v>253</v>
+      </c>
+      <c r="I54" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9">
+      <c r="A55" t="s">
+        <v>37</v>
+      </c>
+      <c r="B55" t="s">
+        <v>40</v>
+      </c>
+      <c r="C55" t="s">
+        <v>76</v>
+      </c>
+      <c r="D55">
+        <v>0.8260869565217391</v>
+      </c>
+      <c r="E55">
+        <v>0.7786561264822134</v>
+      </c>
+      <c r="F55">
+        <v>0.8735177865612648</v>
+      </c>
+      <c r="G55">
+        <v>253</v>
+      </c>
+      <c r="H55">
+        <v>253</v>
+      </c>
+      <c r="I55" t="s">
+        <v>78</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:N55"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -1878,43 +3502,43 @@
         <v>62</v>
       </c>
       <c r="B1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C1" t="s">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="D1" t="s">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="E1" t="s">
+        <v>81</v>
+      </c>
+      <c r="F1" t="s">
+        <v>82</v>
+      </c>
+      <c r="G1" t="s">
+        <v>83</v>
+      </c>
+      <c r="H1" t="s">
         <v>66</v>
       </c>
-      <c r="F1" t="s">
+      <c r="I1" t="s">
         <v>67</v>
       </c>
-      <c r="G1" t="s">
-        <v>68</v>
-      </c>
-      <c r="H1" t="s">
-        <v>69</v>
-      </c>
-      <c r="I1" t="s">
-        <v>70</v>
-      </c>
       <c r="J1" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="K1" t="s">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="L1" t="s">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="M1" t="s">
-        <v>74</v>
+        <v>87</v>
       </c>
       <c r="N1" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2" spans="1:14">
@@ -1922,7 +3546,7 @@
         <v>35</v>
       </c>
       <c r="B2" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C2" t="s">
         <v>38</v>
@@ -1960,7 +3584,7 @@
         <v>35</v>
       </c>
       <c r="B3" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="C3" t="s">
         <v>38</v>
@@ -2004,7 +3628,7 @@
         <v>35</v>
       </c>
       <c r="B4" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C4" t="s">
         <v>38</v>
@@ -2048,7 +3672,7 @@
         <v>35</v>
       </c>
       <c r="B5" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="C5" t="s">
         <v>38</v>
@@ -2092,7 +3716,7 @@
         <v>35</v>
       </c>
       <c r="B6" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C6" t="s">
         <v>38</v>
@@ -2136,7 +3760,7 @@
         <v>35</v>
       </c>
       <c r="B7" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="C7" t="s">
         <v>38</v>
@@ -2180,7 +3804,7 @@
         <v>35</v>
       </c>
       <c r="B8" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C8" t="s">
         <v>38</v>
@@ -2218,7 +3842,7 @@
         <v>35</v>
       </c>
       <c r="B9" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="C9" t="s">
         <v>38</v>
@@ -2262,7 +3886,7 @@
         <v>35</v>
       </c>
       <c r="B10" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C10" t="s">
         <v>38</v>
@@ -2306,7 +3930,7 @@
         <v>35</v>
       </c>
       <c r="B11" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="C11" t="s">
         <v>38</v>
@@ -2350,7 +3974,7 @@
         <v>35</v>
       </c>
       <c r="B12" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C12" t="s">
         <v>38</v>
@@ -2394,7 +4018,7 @@
         <v>35</v>
       </c>
       <c r="B13" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="C13" t="s">
         <v>38</v>
@@ -2438,7 +4062,7 @@
         <v>35</v>
       </c>
       <c r="B14" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C14" t="s">
         <v>39</v>
@@ -2476,7 +4100,7 @@
         <v>35</v>
       </c>
       <c r="B15" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="C15" t="s">
         <v>39</v>
@@ -2520,7 +4144,7 @@
         <v>35</v>
       </c>
       <c r="B16" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C16" t="s">
         <v>39</v>
@@ -2564,7 +4188,7 @@
         <v>35</v>
       </c>
       <c r="B17" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="C17" t="s">
         <v>39</v>
@@ -2608,7 +4232,7 @@
         <v>35</v>
       </c>
       <c r="B18" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C18" t="s">
         <v>39</v>
@@ -2652,7 +4276,7 @@
         <v>35</v>
       </c>
       <c r="B19" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="C19" t="s">
         <v>39</v>
@@ -2696,7 +4320,7 @@
         <v>36</v>
       </c>
       <c r="B20" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C20" t="s">
         <v>38</v>
@@ -2723,7 +4347,7 @@
         <v>0.7589783551323271</v>
       </c>
       <c r="M20" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="N20">
         <v>0.7589783551323271</v>
@@ -2734,7 +4358,7 @@
         <v>36</v>
       </c>
       <c r="B21" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="C21" t="s">
         <v>38</v>
@@ -2772,7 +4396,7 @@
         <v>36</v>
       </c>
       <c r="B22" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C22" t="s">
         <v>38</v>
@@ -2810,7 +4434,7 @@
         <v>36</v>
       </c>
       <c r="B23" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="C23" t="s">
         <v>38</v>
@@ -2837,7 +4461,7 @@
         <v>1</v>
       </c>
       <c r="M23" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="N23">
         <v>1</v>
@@ -2848,7 +4472,7 @@
         <v>36</v>
       </c>
       <c r="B24" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C24" t="s">
         <v>38</v>
@@ -2875,7 +4499,7 @@
         <v>0.8311704095417624</v>
       </c>
       <c r="M24" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="N24">
         <v>0.8311704095417624</v>
@@ -2886,7 +4510,7 @@
         <v>36</v>
       </c>
       <c r="B25" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="C25" t="s">
         <v>38</v>
@@ -2913,7 +4537,7 @@
         <v>1</v>
       </c>
       <c r="M25" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="N25">
         <v>1</v>
@@ -2924,7 +4548,7 @@
         <v>36</v>
       </c>
       <c r="B26" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C26" t="s">
         <v>38</v>
@@ -2951,7 +4575,7 @@
         <v>0.003869222643548615</v>
       </c>
       <c r="M26" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="N26">
         <v>0.01160766793064584</v>
@@ -2962,7 +4586,7 @@
         <v>36</v>
       </c>
       <c r="B27" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="C27" t="s">
         <v>38</v>
@@ -3000,7 +4624,7 @@
         <v>36</v>
       </c>
       <c r="B28" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C28" t="s">
         <v>38</v>
@@ -3038,7 +4662,7 @@
         <v>36</v>
       </c>
       <c r="B29" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="C29" t="s">
         <v>38</v>
@@ -3065,7 +4689,7 @@
         <v>0.6055766163353462</v>
       </c>
       <c r="M29" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="N29">
         <v>1</v>
@@ -3076,7 +4700,7 @@
         <v>36</v>
       </c>
       <c r="B30" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C30" t="s">
         <v>38</v>
@@ -3103,7 +4727,7 @@
         <v>0.02585758046344289</v>
       </c>
       <c r="M30" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="N30">
         <v>0.05171516092688578</v>
@@ -3114,7 +4738,7 @@
         <v>36</v>
       </c>
       <c r="B31" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="C31" t="s">
         <v>38</v>
@@ -3141,7 +4765,7 @@
         <v>0.02373851525005458</v>
       </c>
       <c r="M31" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="N31">
         <v>0.04747703050010915</v>
@@ -3152,7 +4776,7 @@
         <v>36</v>
       </c>
       <c r="B32" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C32" t="s">
         <v>39</v>
@@ -3179,7 +4803,7 @@
         <v>0.009812492570670151</v>
       </c>
       <c r="M32" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="N32">
         <v>0.0196249851413403</v>
@@ -3190,7 +4814,7 @@
         <v>36</v>
       </c>
       <c r="B33" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="C33" t="s">
         <v>39</v>
@@ -3228,7 +4852,7 @@
         <v>36</v>
       </c>
       <c r="B34" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C34" t="s">
         <v>39</v>
@@ -3266,7 +4890,7 @@
         <v>36</v>
       </c>
       <c r="B35" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="C35" t="s">
         <v>39</v>
@@ -3293,7 +4917,7 @@
         <v>0.8025873486341526</v>
       </c>
       <c r="M35" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="N35">
         <v>1</v>
@@ -3304,7 +4928,7 @@
         <v>36</v>
       </c>
       <c r="B36" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C36" t="s">
         <v>39</v>
@@ -3331,7 +4955,7 @@
         <v>0.01480610912734845</v>
       </c>
       <c r="M36" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="N36">
         <v>0.03878637069516434</v>
@@ -3342,7 +4966,7 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="C37" t="s">
         <v>39</v>
@@ -3369,7 +4993,7 @@
         <v>0.02227097895923274</v>
       </c>
       <c r="M37" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="N37">
         <v>0.04454195791846547</v>
@@ -3380,7 +5004,7 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C38" t="s">
         <v>38</v>
@@ -3407,7 +5031,7 @@
         <v>0.1467487068347569</v>
       </c>
       <c r="M38" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="N38">
         <v>0.1467487068347569</v>
@@ -3418,7 +5042,7 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="C39" t="s">
         <v>38</v>
@@ -3456,7 +5080,7 @@
         <v>37</v>
       </c>
       <c r="B40" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C40" t="s">
         <v>38</v>
@@ -3494,7 +5118,7 @@
         <v>37</v>
       </c>
       <c r="B41" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="C41" t="s">
         <v>38</v>
@@ -3521,7 +5145,7 @@
         <v>0.6463551955394902</v>
       </c>
       <c r="M41" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="N41">
         <v>0.6463551955394902</v>
@@ -3532,7 +5156,7 @@
         <v>37</v>
       </c>
       <c r="B42" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C42" t="s">
         <v>38</v>
@@ -3559,7 +5183,7 @@
         <v>0.6276258050283593</v>
       </c>
       <c r="M42" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="N42">
         <v>0.8501067391385259</v>
@@ -3570,7 +5194,7 @@
         <v>37</v>
       </c>
       <c r="B43" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="C43" t="s">
         <v>38</v>
@@ -3597,7 +5221,7 @@
         <v>1</v>
       </c>
       <c r="M43" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="N43">
         <v>1</v>
@@ -3608,7 +5232,7 @@
         <v>37</v>
       </c>
       <c r="B44" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C44" t="s">
         <v>38</v>
@@ -3635,7 +5259,7 @@
         <v>0.003403025345125086</v>
       </c>
       <c r="M44" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="N44">
         <v>0.01020907603537526</v>
@@ -3646,7 +5270,7 @@
         <v>37</v>
       </c>
       <c r="B45" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="C45" t="s">
         <v>38</v>
@@ -3684,7 +5308,7 @@
         <v>37</v>
       </c>
       <c r="B46" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C46" t="s">
         <v>38</v>
@@ -3722,7 +5346,7 @@
         <v>37</v>
       </c>
       <c r="B47" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="C47" t="s">
         <v>38</v>
@@ -3749,7 +5373,7 @@
         <v>0.2109029260566068</v>
       </c>
       <c r="M47" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="N47">
         <v>0.6327087781698203</v>
@@ -3760,7 +5384,7 @@
         <v>37</v>
       </c>
       <c r="B48" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C48" t="s">
         <v>38</v>
@@ -3787,7 +5411,7 @@
         <v>0.8501067391385259</v>
       </c>
       <c r="M48" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="N48">
         <v>0.8501067391385259</v>
@@ -3798,7 +5422,7 @@
         <v>37</v>
       </c>
       <c r="B49" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="C49" t="s">
         <v>38</v>
@@ -3825,7 +5449,7 @@
         <v>0.2626182904425174</v>
       </c>
       <c r="M49" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="N49">
         <v>0.5252365808850348</v>
@@ -3836,7 +5460,7 @@
         <v>37</v>
       </c>
       <c r="B50" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C50" t="s">
         <v>39</v>
@@ -3863,7 +5487,7 @@
         <v>0.04866005335540764</v>
       </c>
       <c r="M50" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="N50">
         <v>0.09732010671081527</v>
@@ -3874,7 +5498,7 @@
         <v>37</v>
       </c>
       <c r="B51" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="C51" t="s">
         <v>39</v>
@@ -3912,7 +5536,7 @@
         <v>37</v>
       </c>
       <c r="B52" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C52" t="s">
         <v>39</v>
@@ -3950,7 +5574,7 @@
         <v>37</v>
       </c>
       <c r="B53" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="C53" t="s">
         <v>39</v>
@@ -3977,7 +5601,7 @@
         <v>0.4795001221869534</v>
       </c>
       <c r="M53" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="N53">
         <v>0.6463551955394902</v>
@@ -3988,7 +5612,7 @@
         <v>37</v>
       </c>
       <c r="B54" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C54" t="s">
         <v>39</v>
@@ -4015,7 +5639,7 @@
         <v>0.4576140668763148</v>
       </c>
       <c r="M54" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="N54">
         <v>0.8501067391385259</v>
@@ -4026,7 +5650,7 @@
         <v>37</v>
       </c>
       <c r="B55" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="C55" t="s">
         <v>39</v>
@@ -4053,7 +5677,7 @@
         <v>0.2432427057426535</v>
       </c>
       <c r="M55" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="N55">
         <v>0.486485411485307</v>
@@ -4064,7 +5688,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:P4"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -4074,49 +5698,49 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="C1" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="D1" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="E1" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="F1" t="s">
-        <v>88</v>
+        <v>68</v>
       </c>
       <c r="G1" t="s">
-        <v>89</v>
+        <v>69</v>
       </c>
       <c r="H1" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="I1" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="J1" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="K1" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="L1" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="M1" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="N1" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="O1" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="P1" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
     </row>
     <row r="2" spans="1:16">
@@ -4124,16 +5748,16 @@
         <v>35</v>
       </c>
       <c r="B2" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="C2" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="D2" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="E2" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="F2">
         <v>516</v>
@@ -4157,16 +5781,16 @@
         <v>42</v>
       </c>
       <c r="M2" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="N2" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="O2" t="b">
         <v>0</v>
       </c>
       <c r="P2" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:16">
@@ -4174,16 +5798,16 @@
         <v>36</v>
       </c>
       <c r="B3" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="C3" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="D3" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="E3" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="F3">
         <v>263</v>
@@ -4207,16 +5831,16 @@
         <v>42</v>
       </c>
       <c r="M3" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="N3" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="O3" t="b">
         <v>0</v>
       </c>
       <c r="P3" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
     </row>
     <row r="4" spans="1:16">
@@ -4224,16 +5848,16 @@
         <v>37</v>
       </c>
       <c r="B4" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="C4" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="D4" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="E4" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="F4">
         <v>253</v>
@@ -4257,16 +5881,16 @@
         <v>42</v>
       </c>
       <c r="M4" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="N4" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="O4" t="b">
         <v>0</v>
       </c>
       <c r="P4" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>

</xml_diff>